<commit_message>
feat: 6-sheet Excel template + round-based slot parsing (cmd_029+030)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/template/kumano_draft_template.xlsx
+++ b/public/template/kumano_draft_template.xlsx
@@ -3,10 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="枠数設定" sheetId="1" r:id="rId1"/>
-    <sheet name="新入生" sheetId="2" r:id="rId2"/>
-    <sheet name="上回生" sheetId="3" r:id="rId3"/>
-    <sheet name="臨時" sheetId="4" r:id="rId4"/>
+    <sheet name="新入生枠数設定" sheetId="1" r:id="rId1"/>
+    <sheet name="上回生枠数設定" sheetId="2" r:id="rId2"/>
+    <sheet name="臨キャパ枠数設定" sheetId="3" r:id="rId3"/>
+    <sheet name="新入生一覧" sheetId="4" r:id="rId4"/>
+    <sheet name="上回生一覧" sheetId="5" r:id="rId5"/>
+    <sheet name="臨キャパ一覧" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -400,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D10"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -424,13 +426,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Aブロック</v>
+        <v>A1</v>
       </c>
       <c r="B2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D2">
         <v>2</v>
@@ -438,26 +440,485 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Bブロック</v>
+        <v>A2</v>
       </c>
       <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>A3</v>
+      </c>
+      <c r="B4">
+        <v>6</v>
+      </c>
+      <c r="C4">
         <v>4</v>
       </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
+      <c r="D4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>A4</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>B12</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>B3</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>B4</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>C12</v>
+      </c>
+      <c r="B9">
+        <v>3</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>C34</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D10"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ブロック名</v>
+      </c>
+      <c r="B1" t="str">
+        <v>合計</v>
+      </c>
+      <c r="C1" t="str">
+        <v>第1巡枠数</v>
+      </c>
+      <c r="D1" t="str">
+        <v>第2巡枠数</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>A1</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>A2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>A3</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>A4</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>B12</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>B3</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>B4</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>C12</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>C34</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D10"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ブロック名</v>
+      </c>
+      <c r="B1" t="str">
+        <v>合計</v>
+      </c>
+      <c r="C1" t="str">
+        <v>第1巡枠数</v>
+      </c>
+      <c r="D1" t="str">
+        <v>第2巡枠数</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>A1</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>A2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>A3</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>A4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>B12</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>B3</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>B4</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>C12</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>C34</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B4"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>番号</v>
+      </c>
+      <c r="B1" t="str">
+        <v>氏名</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>山田太郎</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>佐藤花子</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>鈴木一郎</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
   <cols>
@@ -470,7 +931,7 @@
         <v>番号</v>
       </c>
       <c r="B1" t="str">
-        <v>名前</v>
+        <v>氏名</v>
       </c>
     </row>
     <row r="2">
@@ -478,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>山田太郎</v>
+        <v>田中二郎</v>
       </c>
     </row>
     <row r="3">
@@ -486,7 +947,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>佐藤花子</v>
+        <v>高橋三郎</v>
       </c>
     </row>
   </sheetData>
@@ -496,9 +957,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -509,7 +970,7 @@
         <v>番号</v>
       </c>
       <c r="B1" t="str">
-        <v>名前</v>
+        <v>氏名</v>
       </c>
     </row>
     <row r="2">
@@ -517,43 +978,20 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>鈴木一郎</v>
+        <v>渡辺四郎</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>伊藤五郎</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
-  <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>番号</v>
-      </c>
-      <c r="B1" t="str">
-        <v>名前</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>高橋次郎</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>